<commit_message>
fix ILP model (Closes #1)
</commit_message>
<xml_diff>
--- a/data/df_compatibility_matrix.xlsx
+++ b/data/df_compatibility_matrix.xlsx
@@ -1,20 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Q:\VitaliteNB\Aide à la décision\IntelligencePredictive_IA\3_Optimisation Transfers\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CD4E8C7-6A20-40BE-B38A-D1A1DC5A008E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$197</definedName>
+  </definedNames>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="18">
   <si>
     <t>origin</t>
   </si>
@@ -66,12 +75,15 @@
   <si>
     <t>SOINS INTERMEDIAIRES</t>
   </si>
+  <si>
+    <t>3B-MERE ENFANT</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,13 +146,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -178,7 +198,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -212,6 +232,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -246,9 +267,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -421,11 +443,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:C197"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -436,9 +463,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -447,7 +474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -458,7 +485,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -469,7 +496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -480,7 +507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -491,7 +518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -502,7 +529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -513,7 +540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -524,7 +551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -535,7 +562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -546,7 +573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -557,7 +584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -568,7 +595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -579,7 +606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -590,9 +617,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
         <v>4</v>
@@ -601,7 +628,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -612,7 +639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -623,7 +650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -634,7 +661,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -645,7 +672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -656,7 +683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -667,7 +694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -678,7 +705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -689,7 +716,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -700,7 +727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -711,7 +738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>14</v>
       </c>
@@ -722,7 +749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>15</v>
       </c>
@@ -733,7 +760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -744,9 +771,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B30" t="s">
         <v>5</v>
@@ -755,7 +782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -766,7 +793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>5</v>
       </c>
@@ -777,7 +804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>6</v>
       </c>
@@ -788,7 +815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>7</v>
       </c>
@@ -799,7 +826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -810,7 +837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>9</v>
       </c>
@@ -821,7 +848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>10</v>
       </c>
@@ -832,7 +859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>11</v>
       </c>
@@ -843,7 +870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>12</v>
       </c>
@@ -854,7 +881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -865,7 +892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>14</v>
       </c>
@@ -876,7 +903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>15</v>
       </c>
@@ -887,7 +914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>16</v>
       </c>
@@ -898,9 +925,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B44" t="s">
         <v>6</v>
@@ -909,7 +936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>4</v>
       </c>
@@ -920,7 +947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>5</v>
       </c>
@@ -931,7 +958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>6</v>
       </c>
@@ -942,7 +969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>7</v>
       </c>
@@ -953,7 +980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>8</v>
       </c>
@@ -964,7 +991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>9</v>
       </c>
@@ -975,7 +1002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>10</v>
       </c>
@@ -986,7 +1013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>11</v>
       </c>
@@ -997,7 +1024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>12</v>
       </c>
@@ -1008,7 +1035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>13</v>
       </c>
@@ -1019,7 +1046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>14</v>
       </c>
@@ -1030,7 +1057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>15</v>
       </c>
@@ -1041,7 +1068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>16</v>
       </c>
@@ -1052,9 +1079,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B58" t="s">
         <v>7</v>
@@ -1063,7 +1090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>4</v>
       </c>
@@ -1074,7 +1101,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>5</v>
       </c>
@@ -1085,7 +1112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>6</v>
       </c>
@@ -1096,7 +1123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
+    <row r="62" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>7</v>
       </c>
@@ -1107,7 +1134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -1118,7 +1145,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>9</v>
       </c>
@@ -1129,7 +1156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>10</v>
       </c>
@@ -1140,7 +1167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>11</v>
       </c>
@@ -1151,7 +1178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>12</v>
       </c>
@@ -1162,7 +1189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -1173,7 +1200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>14</v>
       </c>
@@ -1184,7 +1211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>15</v>
       </c>
@@ -1195,7 +1222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>16</v>
       </c>
@@ -1206,9 +1233,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B72" t="s">
         <v>8</v>
@@ -1217,7 +1244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>4</v>
       </c>
@@ -1228,7 +1255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>5</v>
       </c>
@@ -1239,7 +1266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>6</v>
       </c>
@@ -1250,7 +1277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:3">
+    <row r="76" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>7</v>
       </c>
@@ -1261,7 +1288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:3">
+    <row r="77" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>8</v>
       </c>
@@ -1272,7 +1299,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:3">
+    <row r="78" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>9</v>
       </c>
@@ -1283,7 +1310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:3">
+    <row r="79" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>10</v>
       </c>
@@ -1294,7 +1321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:3">
+    <row r="80" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>11</v>
       </c>
@@ -1305,7 +1332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:3">
+    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>12</v>
       </c>
@@ -1316,7 +1343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:3">
+    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>13</v>
       </c>
@@ -1327,7 +1354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>14</v>
       </c>
@@ -1338,7 +1365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>15</v>
       </c>
@@ -1349,7 +1376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:3">
+    <row r="85" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>16</v>
       </c>
@@ -1360,9 +1387,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B86" t="s">
         <v>9</v>
@@ -1371,7 +1398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>4</v>
       </c>
@@ -1382,7 +1409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>5</v>
       </c>
@@ -1393,7 +1420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>6</v>
       </c>
@@ -1404,7 +1431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>7</v>
       </c>
@@ -1415,7 +1442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>8</v>
       </c>
@@ -1426,7 +1453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>9</v>
       </c>
@@ -1437,7 +1464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>10</v>
       </c>
@@ -1448,7 +1475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>11</v>
       </c>
@@ -1459,7 +1486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>12</v>
       </c>
@@ -1470,7 +1497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>13</v>
       </c>
@@ -1481,7 +1508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:3">
+    <row r="97" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>14</v>
       </c>
@@ -1492,7 +1519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:3">
+    <row r="98" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>15</v>
       </c>
@@ -1503,7 +1530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>16</v>
       </c>
@@ -1514,9 +1541,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B100" t="s">
         <v>10</v>
@@ -1525,7 +1552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>4</v>
       </c>
@@ -1536,7 +1563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>5</v>
       </c>
@@ -1547,7 +1574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>6</v>
       </c>
@@ -1558,7 +1585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>7</v>
       </c>
@@ -1569,7 +1596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>8</v>
       </c>
@@ -1580,7 +1607,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>9</v>
       </c>
@@ -1591,7 +1618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>10</v>
       </c>
@@ -1602,7 +1629,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>11</v>
       </c>
@@ -1613,7 +1640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>12</v>
       </c>
@@ -1624,7 +1651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>13</v>
       </c>
@@ -1635,7 +1662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:3">
+    <row r="111" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>14</v>
       </c>
@@ -1646,7 +1673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>15</v>
       </c>
@@ -1657,7 +1684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:3">
+    <row r="113" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>16</v>
       </c>
@@ -1668,9 +1695,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:3">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B114" t="s">
         <v>11</v>
@@ -1679,7 +1706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:3">
+    <row r="115" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>4</v>
       </c>
@@ -1690,7 +1717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:3">
+    <row r="116" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>5</v>
       </c>
@@ -1701,7 +1728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:3">
+    <row r="117" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>6</v>
       </c>
@@ -1712,7 +1739,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:3">
+    <row r="118" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>7</v>
       </c>
@@ -1723,7 +1750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:3">
+    <row r="119" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>8</v>
       </c>
@@ -1734,7 +1761,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:3">
+    <row r="120" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>9</v>
       </c>
@@ -1745,7 +1772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:3">
+    <row r="121" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>10</v>
       </c>
@@ -1756,7 +1783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:3">
+    <row r="122" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>11</v>
       </c>
@@ -1767,7 +1794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:3">
+    <row r="123" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>12</v>
       </c>
@@ -1778,7 +1805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:3">
+    <row r="124" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>13</v>
       </c>
@@ -1789,7 +1816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:3">
+    <row r="125" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>14</v>
       </c>
@@ -1800,7 +1827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:3">
+    <row r="126" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>15</v>
       </c>
@@ -1811,7 +1838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:3">
+    <row r="127" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>16</v>
       </c>
@@ -1822,9 +1849,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:3">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B128" t="s">
         <v>12</v>
@@ -1833,7 +1860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:3">
+    <row r="129" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>4</v>
       </c>
@@ -1844,7 +1871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:3">
+    <row r="130" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>5</v>
       </c>
@@ -1855,7 +1882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:3">
+    <row r="131" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>6</v>
       </c>
@@ -1866,7 +1893,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:3">
+    <row r="132" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>7</v>
       </c>
@@ -1877,7 +1904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:3">
+    <row r="133" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>8</v>
       </c>
@@ -1888,7 +1915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:3">
+    <row r="134" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>9</v>
       </c>
@@ -1899,7 +1926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:3">
+    <row r="135" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>10</v>
       </c>
@@ -1910,7 +1937,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:3">
+    <row r="136" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>11</v>
       </c>
@@ -1921,7 +1948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:3">
+    <row r="137" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>12</v>
       </c>
@@ -1932,7 +1959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:3">
+    <row r="138" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>13</v>
       </c>
@@ -1943,7 +1970,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:3">
+    <row r="139" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>14</v>
       </c>
@@ -1954,7 +1981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:3">
+    <row r="140" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>15</v>
       </c>
@@ -1965,7 +1992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:3">
+    <row r="141" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>16</v>
       </c>
@@ -1976,9 +2003,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:3">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B142" t="s">
         <v>13</v>
@@ -1987,7 +2014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:3">
+    <row r="143" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>4</v>
       </c>
@@ -1998,7 +2025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:3">
+    <row r="144" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>5</v>
       </c>
@@ -2009,7 +2036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:3">
+    <row r="145" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>6</v>
       </c>
@@ -2020,7 +2047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:3">
+    <row r="146" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>7</v>
       </c>
@@ -2031,7 +2058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:3">
+    <row r="147" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>8</v>
       </c>
@@ -2042,7 +2069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:3">
+    <row r="148" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>9</v>
       </c>
@@ -2053,7 +2080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:3">
+    <row r="149" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>10</v>
       </c>
@@ -2064,7 +2091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:3">
+    <row r="150" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>11</v>
       </c>
@@ -2075,7 +2102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:3">
+    <row r="151" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>12</v>
       </c>
@@ -2086,7 +2113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:3">
+    <row r="152" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>13</v>
       </c>
@@ -2097,7 +2124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:3">
+    <row r="153" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>14</v>
       </c>
@@ -2108,7 +2135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:3">
+    <row r="154" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>15</v>
       </c>
@@ -2119,7 +2146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:3">
+    <row r="155" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>16</v>
       </c>
@@ -2130,9 +2157,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:3">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B156" t="s">
         <v>14</v>
@@ -2141,7 +2168,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:3">
+    <row r="157" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>4</v>
       </c>
@@ -2152,7 +2179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:3">
+    <row r="158" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>5</v>
       </c>
@@ -2163,7 +2190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:3">
+    <row r="159" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>6</v>
       </c>
@@ -2174,7 +2201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:3">
+    <row r="160" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>7</v>
       </c>
@@ -2185,7 +2212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:3">
+    <row r="161" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>8</v>
       </c>
@@ -2196,7 +2223,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:3">
+    <row r="162" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>9</v>
       </c>
@@ -2207,7 +2234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:3">
+    <row r="163" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>10</v>
       </c>
@@ -2218,7 +2245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:3">
+    <row r="164" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>11</v>
       </c>
@@ -2229,7 +2256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:3">
+    <row r="165" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>12</v>
       </c>
@@ -2240,7 +2267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:3">
+    <row r="166" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>13</v>
       </c>
@@ -2251,7 +2278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:3">
+    <row r="167" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>14</v>
       </c>
@@ -2262,7 +2289,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:3">
+    <row r="168" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>15</v>
       </c>
@@ -2273,7 +2300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:3">
+    <row r="169" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>16</v>
       </c>
@@ -2284,9 +2311,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:3">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B170" t="s">
         <v>15</v>
@@ -2295,7 +2322,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:3">
+    <row r="171" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>4</v>
       </c>
@@ -2306,7 +2333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:3">
+    <row r="172" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>5</v>
       </c>
@@ -2317,7 +2344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:3">
+    <row r="173" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>6</v>
       </c>
@@ -2328,7 +2355,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:3">
+    <row r="174" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>7</v>
       </c>
@@ -2339,7 +2366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:3">
+    <row r="175" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>8</v>
       </c>
@@ -2350,7 +2377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:3">
+    <row r="176" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>9</v>
       </c>
@@ -2361,7 +2388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:3">
+    <row r="177" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>10</v>
       </c>
@@ -2372,7 +2399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="1:3">
+    <row r="178" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>11</v>
       </c>
@@ -2383,7 +2410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:3">
+    <row r="179" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>12</v>
       </c>
@@ -2394,7 +2421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="1:3">
+    <row r="180" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>13</v>
       </c>
@@ -2405,7 +2432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="1:3">
+    <row r="181" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>14</v>
       </c>
@@ -2416,7 +2443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:3">
+    <row r="182" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>15</v>
       </c>
@@ -2427,7 +2454,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:3">
+    <row r="183" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>16</v>
       </c>
@@ -2438,9 +2465,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:3">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B184" t="s">
         <v>16</v>
@@ -2449,7 +2476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:3">
+    <row r="185" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>4</v>
       </c>
@@ -2460,7 +2487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:3">
+    <row r="186" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>5</v>
       </c>
@@ -2471,7 +2498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:3">
+    <row r="187" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>6</v>
       </c>
@@ -2482,7 +2509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:3">
+    <row r="188" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>7</v>
       </c>
@@ -2493,7 +2520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:3">
+    <row r="189" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>8</v>
       </c>
@@ -2504,7 +2531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:3">
+    <row r="190" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>9</v>
       </c>
@@ -2515,7 +2542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:3">
+    <row r="191" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>10</v>
       </c>
@@ -2526,7 +2553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:3">
+    <row r="192" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>11</v>
       </c>
@@ -2537,7 +2564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:3">
+    <row r="193" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>12</v>
       </c>
@@ -2548,7 +2575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:3">
+    <row r="194" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>13</v>
       </c>
@@ -2559,7 +2586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:3">
+    <row r="195" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>14</v>
       </c>
@@ -2570,7 +2597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:3">
+    <row r="196" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>15</v>
       </c>
@@ -2581,7 +2608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:3">
+    <row r="197" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>16</v>
       </c>
@@ -2593,6 +2620,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C197" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="3B-GYNECO/OBS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
cleaned files and git ignore added
</commit_message>
<xml_diff>
--- a/data/df_compatibility_matrix.xlsx
+++ b/data/df_compatibility_matrix.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Q:\VitaliteNB\Aide à la décision\IntelligencePredictive_IA\3_Optimisation Transfers\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF0BB890-634B-464C-BF0E-5DA0FE2D9F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFBE79D5-D0C1-43A2-855C-90C7C6B68EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{682C894F-F8B8-46AB-B924-76032B5586F1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{682C894F-F8B8-46AB-B924-76032B5586F1}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1'!$A$1:$C$197</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="18">
   <si>
     <t>origin</t>
   </si>
@@ -71,6 +74,9 @@
   </si>
   <si>
     <t>4CSI</t>
+  </si>
+  <si>
+    <t>SINTER</t>
   </si>
 </sst>
 </file>
@@ -932,9 +938,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{613290DD-B4F8-45A7-BC6C-8C365265D4DA}">
   <dimension ref="A1:C197"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -945,7 +951,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -956,7 +962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -967,7 +973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -978,7 +984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -989,7 +995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -1000,7 +1006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1011,7 +1017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1022,7 +1028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1033,7 +1039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1044,7 +1050,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1055,7 +1061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1066,7 +1072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -1077,7 +1083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -1088,9 +1094,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
         <v>3</v>
@@ -1099,7 +1105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>3</v>
       </c>
@@ -1110,7 +1116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -1121,7 +1127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -1132,7 +1138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -1143,7 +1149,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -1154,7 +1160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -1165,7 +1171,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -1176,7 +1182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -1187,7 +1193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -1198,7 +1204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -1209,7 +1215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -1220,7 +1226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>14</v>
       </c>
@@ -1231,7 +1237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>15</v>
       </c>
@@ -1242,9 +1248,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B29" t="s">
         <v>4</v>
@@ -1253,7 +1259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>3</v>
       </c>
@@ -1264,7 +1270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -1275,7 +1281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>5</v>
       </c>
@@ -1286,7 +1292,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>6</v>
       </c>
@@ -1297,7 +1303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>7</v>
       </c>
@@ -1308,7 +1314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -1319,7 +1325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>9</v>
       </c>
@@ -1330,7 +1336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>10</v>
       </c>
@@ -1341,7 +1347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>11</v>
       </c>
@@ -1352,7 +1358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>12</v>
       </c>
@@ -1363,7 +1369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -1374,7 +1380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>14</v>
       </c>
@@ -1385,7 +1391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>15</v>
       </c>
@@ -1396,9 +1402,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B43" t="s">
         <v>5</v>
@@ -1407,7 +1413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -1418,7 +1424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>4</v>
       </c>
@@ -1429,7 +1435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>5</v>
       </c>
@@ -1440,7 +1446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>6</v>
       </c>
@@ -1451,7 +1457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>7</v>
       </c>
@@ -1462,7 +1468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>8</v>
       </c>
@@ -1473,7 +1479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>9</v>
       </c>
@@ -1484,7 +1490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>10</v>
       </c>
@@ -1495,7 +1501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>11</v>
       </c>
@@ -1506,7 +1512,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>12</v>
       </c>
@@ -1517,7 +1523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>13</v>
       </c>
@@ -1528,7 +1534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>14</v>
       </c>
@@ -1539,7 +1545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>15</v>
       </c>
@@ -1550,9 +1556,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B57" t="s">
         <v>6</v>
@@ -1561,7 +1567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>3</v>
       </c>
@@ -1572,7 +1578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>4</v>
       </c>
@@ -1583,7 +1589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>5</v>
       </c>
@@ -1594,7 +1600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>6</v>
       </c>
@@ -1605,7 +1611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>7</v>
       </c>
@@ -1616,7 +1622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -1627,7 +1633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>9</v>
       </c>
@@ -1638,7 +1644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>10</v>
       </c>
@@ -1649,7 +1655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>11</v>
       </c>
@@ -1660,7 +1666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>12</v>
       </c>
@@ -1671,7 +1677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -1682,7 +1688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>14</v>
       </c>
@@ -1693,7 +1699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>15</v>
       </c>
@@ -1704,9 +1710,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B71" t="s">
         <v>7</v>
@@ -1715,7 +1721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>3</v>
       </c>
@@ -1726,7 +1732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>4</v>
       </c>
@@ -1737,7 +1743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>5</v>
       </c>
@@ -1748,7 +1754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>6</v>
       </c>
@@ -1759,7 +1765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>7</v>
       </c>
@@ -1770,7 +1776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>8</v>
       </c>
@@ -1781,7 +1787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>9</v>
       </c>
@@ -1792,7 +1798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>10</v>
       </c>
@@ -1803,7 +1809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>11</v>
       </c>
@@ -1814,7 +1820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>12</v>
       </c>
@@ -1825,7 +1831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>13</v>
       </c>
@@ -1836,7 +1842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>14</v>
       </c>
@@ -1847,7 +1853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>15</v>
       </c>
@@ -1858,9 +1864,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B85" t="s">
         <v>8</v>
@@ -1869,7 +1875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>3</v>
       </c>
@@ -1880,7 +1886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>4</v>
       </c>
@@ -1891,7 +1897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>5</v>
       </c>
@@ -1902,7 +1908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>6</v>
       </c>
@@ -1913,7 +1919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>7</v>
       </c>
@@ -1924,7 +1930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>8</v>
       </c>
@@ -1935,7 +1941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>9</v>
       </c>
@@ -1946,7 +1952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>10</v>
       </c>
@@ -1957,7 +1963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>11</v>
       </c>
@@ -1968,7 +1974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>12</v>
       </c>
@@ -1979,7 +1985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>13</v>
       </c>
@@ -1990,7 +1996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>14</v>
       </c>
@@ -2001,7 +2007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>15</v>
       </c>
@@ -2012,9 +2018,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B99" t="s">
         <v>9</v>
@@ -2023,7 +2029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>3</v>
       </c>
@@ -2034,7 +2040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>4</v>
       </c>
@@ -2045,7 +2051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>5</v>
       </c>
@@ -2056,7 +2062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>6</v>
       </c>
@@ -2067,7 +2073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>7</v>
       </c>
@@ -2078,7 +2084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>8</v>
       </c>
@@ -2089,7 +2095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>9</v>
       </c>
@@ -2100,7 +2106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>10</v>
       </c>
@@ -2111,7 +2117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>11</v>
       </c>
@@ -2122,7 +2128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>12</v>
       </c>
@@ -2133,7 +2139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>13</v>
       </c>
@@ -2144,7 +2150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>14</v>
       </c>
@@ -2155,7 +2161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>15</v>
       </c>
@@ -2166,9 +2172,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B113" t="s">
         <v>10</v>
@@ -2177,7 +2183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>3</v>
       </c>
@@ -2188,7 +2194,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>4</v>
       </c>
@@ -2199,7 +2205,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>5</v>
       </c>
@@ -2210,7 +2216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>6</v>
       </c>
@@ -2221,7 +2227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>7</v>
       </c>
@@ -2232,7 +2238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>8</v>
       </c>
@@ -2243,7 +2249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>9</v>
       </c>
@@ -2254,7 +2260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>10</v>
       </c>
@@ -2265,7 +2271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>11</v>
       </c>
@@ -2276,7 +2282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>12</v>
       </c>
@@ -2287,7 +2293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>13</v>
       </c>
@@ -2298,7 +2304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>14</v>
       </c>
@@ -2309,7 +2315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>15</v>
       </c>
@@ -2320,9 +2326,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B127" t="s">
         <v>11</v>
@@ -2331,7 +2337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>3</v>
       </c>
@@ -2342,7 +2348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>4</v>
       </c>
@@ -2353,7 +2359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>5</v>
       </c>
@@ -2364,7 +2370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>6</v>
       </c>
@@ -2375,7 +2381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>7</v>
       </c>
@@ -2386,7 +2392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>8</v>
       </c>
@@ -2397,7 +2403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>9</v>
       </c>
@@ -2408,7 +2414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>10</v>
       </c>
@@ -2419,7 +2425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>11</v>
       </c>
@@ -2430,7 +2436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>12</v>
       </c>
@@ -2441,7 +2447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>13</v>
       </c>
@@ -2452,7 +2458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>14</v>
       </c>
@@ -2463,7 +2469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>15</v>
       </c>
@@ -2474,9 +2480,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B141" t="s">
         <v>12</v>
@@ -2485,7 +2491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>3</v>
       </c>
@@ -2496,7 +2502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>4</v>
       </c>
@@ -2507,7 +2513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>5</v>
       </c>
@@ -2518,7 +2524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>6</v>
       </c>
@@ -2529,7 +2535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>7</v>
       </c>
@@ -2540,7 +2546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>8</v>
       </c>
@@ -2551,7 +2557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>9</v>
       </c>
@@ -2562,7 +2568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>10</v>
       </c>
@@ -2573,7 +2579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>11</v>
       </c>
@@ -2584,7 +2590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>12</v>
       </c>
@@ -2595,7 +2601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>13</v>
       </c>
@@ -2606,7 +2612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>14</v>
       </c>
@@ -2617,7 +2623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>15</v>
       </c>
@@ -2628,9 +2634,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B155" t="s">
         <v>13</v>
@@ -2639,7 +2645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>3</v>
       </c>
@@ -2650,7 +2656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>4</v>
       </c>
@@ -2661,7 +2667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>5</v>
       </c>
@@ -2672,7 +2678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>6</v>
       </c>
@@ -2683,7 +2689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>7</v>
       </c>
@@ -2694,7 +2700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>8</v>
       </c>
@@ -2705,7 +2711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>9</v>
       </c>
@@ -2716,7 +2722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>10</v>
       </c>
@@ -2727,7 +2733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>11</v>
       </c>
@@ -2738,7 +2744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>12</v>
       </c>
@@ -2749,7 +2755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>13</v>
       </c>
@@ -2760,7 +2766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>14</v>
       </c>
@@ -2771,7 +2777,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>15</v>
       </c>
@@ -2782,9 +2788,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B169" t="s">
         <v>14</v>
@@ -2793,7 +2799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>3</v>
       </c>
@@ -2804,7 +2810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>4</v>
       </c>
@@ -2815,7 +2821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>5</v>
       </c>
@@ -2826,7 +2832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>6</v>
       </c>
@@ -2837,7 +2843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>7</v>
       </c>
@@ -2848,7 +2854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>8</v>
       </c>
@@ -2859,7 +2865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>9</v>
       </c>
@@ -2870,7 +2876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>10</v>
       </c>
@@ -2881,7 +2887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>11</v>
       </c>
@@ -2892,7 +2898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>12</v>
       </c>
@@ -2903,7 +2909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>13</v>
       </c>
@@ -2914,7 +2920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>14</v>
       </c>
@@ -2925,7 +2931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>15</v>
       </c>
@@ -2936,9 +2942,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B183" t="s">
         <v>15</v>
@@ -2947,7 +2953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>3</v>
       </c>
@@ -2958,7 +2964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>4</v>
       </c>
@@ -2969,7 +2975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>5</v>
       </c>
@@ -2980,7 +2986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>6</v>
       </c>
@@ -2991,7 +2997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>7</v>
       </c>
@@ -3002,7 +3008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>8</v>
       </c>
@@ -3013,7 +3019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>9</v>
       </c>
@@ -3024,7 +3030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>10</v>
       </c>
@@ -3035,7 +3041,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>11</v>
       </c>
@@ -3046,7 +3052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>12</v>
       </c>
@@ -3057,7 +3063,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>13</v>
       </c>
@@ -3068,7 +3074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>14</v>
       </c>
@@ -3079,7 +3085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>15</v>
       </c>
@@ -3090,9 +3096,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B197" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
model bug fixed Closes #5
</commit_message>
<xml_diff>
--- a/data/df_compatibility_matrix.xlsx
+++ b/data/df_compatibility_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Q:\VitaliteNB\Aide à la décision\IntelligencePredictive_IA\3_Optimisation Transfers\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFBE79D5-D0C1-43A2-855C-90C7C6B68EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14720523-F62D-470A-96AE-1B41D2BC45A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{682C894F-F8B8-46AB-B924-76032B5586F1}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="17">
   <si>
     <t>origin</t>
   </si>
@@ -71,9 +71,6 @@
   </si>
   <si>
     <t>SCOR</t>
-  </si>
-  <si>
-    <t>4CSI</t>
   </si>
   <si>
     <t>SINTER</t>
@@ -939,6 +936,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{613290DD-B4F8-45A7-BC6C-8C365265D4DA}">
   <dimension ref="A1:C197"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -1096,7 +1097,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" t="s">
         <v>3</v>
@@ -1250,7 +1251,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B29" t="s">
         <v>4</v>
@@ -1404,7 +1405,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B43" t="s">
         <v>5</v>
@@ -1558,7 +1559,7 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B57" t="s">
         <v>6</v>
@@ -1712,7 +1713,7 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B71" t="s">
         <v>7</v>
@@ -1866,7 +1867,7 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B85" t="s">
         <v>8</v>
@@ -2020,7 +2021,7 @@
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B99" t="s">
         <v>9</v>
@@ -2174,7 +2175,7 @@
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B113" t="s">
         <v>10</v>
@@ -2328,7 +2329,7 @@
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B127" t="s">
         <v>11</v>
@@ -2482,7 +2483,7 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B141" t="s">
         <v>12</v>
@@ -2636,7 +2637,7 @@
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B155" t="s">
         <v>13</v>
@@ -2790,7 +2791,7 @@
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B169" t="s">
         <v>14</v>
@@ -2944,7 +2945,7 @@
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B183" t="s">
         <v>15</v>
@@ -3098,7 +3099,7 @@
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B197" t="s">
         <v>16</v>

</xml_diff>